<commit_message>
Refactor notebook and paper builders for improved clarity and functionality
- Updated the `build_notebook` function to reflect the final course paper structure, ensuring all calculations are sourced from formal result files.
- Removed outdated code related to notebook execution and streamlined the notebook creation process.
- Enhanced the `build_paper` function by integrating new metrics from text model evaluations and improving the structure of validation results.
- Adjusted PDF generation to include a cover page and refined formatting for better readability.
- Updated lexicon building to clarify the limitations of sentence-level sentiment accuracy.
- Improved section repair logic to handle local paths more robustly.
</commit_message>
<xml_diff>
--- a/paper/数字一致性审计.xlsx
+++ b/paper/数字一致性审计.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0955076786677384</v>
+        <v>0.09444690550353113</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1887370910306666</v>
+        <v>0.1887716020499765</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10.02172702043578</v>
+        <v>9.905080803459022</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -571,13 +571,73 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>svc_sentiment_cv_accuracy</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>output/results/text_model_evaluation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>svc_policy_stance_cv_accuracy</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.8583333333333333</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>output/results/text_model_evaluation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>svc_policy_direction_cv_accuracy</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.7878787878787878</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>output/results/text_model_evaluation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>svc_topic_cv_macro_f1</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3329096913900582</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>output/results/text_model_evaluation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>manual_validation_rows</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B15" t="n">
         <v>240</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>data/validation/manual_sentence_annotation_filled.xlsx</t>
         </is>

</xml_diff>

<commit_message>
Refactor monetary policy analysis and reporting scripts with localization improvements
- Updated comments and labels in power_analysis.py to include Chinese translations for better accessibility.
- Modified project usage descriptions in pipeline.py for clarity and consistency in terminology.
- Enhanced paper_builder.py by changing font styles and sizes for better readability, and adjusted references to include more recent studies.
- Improved visualization scripts (market_figures.py, result_tables.py, text_figures.py) with updated color schemes and line styles for better visual representation.
- Ensured consistent terminology across the codebase, particularly in relation to the exploratory models and their interactions.
</commit_message>
<xml_diff>
--- a/paper/数字一致性审计.xlsx
+++ b/paper/数字一致性审计.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.09444690550353113</v>
+        <v>0.0955076786677384</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1887716020499765</v>
+        <v>0.1887370910306666</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9.905080803459022</v>
+        <v>10.02172702043578</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: Enhance journal paper generation and auditing tools
- Added document sanitization to replace engineering terms with their Chinese equivalents in the journal paper.
- Implemented normalization of DOCX spacing rules to avoid fixed-spacing tags.
- Updated title formatting in the journal paper to improve presentation.
- Introduced a backup script to archive important files before edits.
- Created a script to build the journal paper from output results, integrating various data sources.
- Developed a paper audit tool to check for forbidden terms and layout discrepancies in the generated PDF.
- Added functionality to render PDFs to PNGs for visual comparison against reference documents.
- Enhanced error handling and reporting in the auditing process.
</commit_message>
<xml_diff>
--- a/paper/数字一致性审计.xlsx
+++ b/paper/数字一致性审计.xlsx
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1631866708367444</v>
+        <v>0.1631866708367445</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.2958333333333333</v>
+        <v>0.2958</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.5303030303030303</v>
+        <v>0.5303</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>

</xml_diff>